<commit_message>
Get repo up to date
Unfortunately lots of junk here to clean up later. I'm just going to commit everything then tidy progressively as-needed.
</commit_message>
<xml_diff>
--- a/data/2025/metadata/data_inventory.xlsx
+++ b/data/2025/metadata/data_inventory.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/drotto/src/jiflr/data/2025/metadata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53DA5416-EEC2-8943-8E6A-D66EABF17990}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D720A247-0A5F-1A41-9810-EC846048D1B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1100" yWindow="880" windowWidth="34900" windowHeight="22500" activeTab="1" xr2:uid="{834A5152-98D4-1D4E-9988-BEC817907187}"/>
+    <workbookView xWindow="1180" yWindow="780" windowWidth="34820" windowHeight="22600" xr2:uid="{834A5152-98D4-1D4E-9988-BEC817907187}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="106">
   <si>
     <t>site_id</t>
   </si>
@@ -160,12 +160,6 @@
     <t>site_type</t>
   </si>
   <si>
-    <t>temperature</t>
-  </si>
-  <si>
-    <t>intensive</t>
-  </si>
-  <si>
     <t>There was a 0 cm sensor here that failed before being deployed</t>
   </si>
   <si>
@@ -178,9 +172,6 @@
     <t>Missing 0m data file</t>
   </si>
   <si>
-    <t>camp</t>
-  </si>
-  <si>
     <t>C17</t>
   </si>
   <si>
@@ -205,9 +196,6 @@
     <t>C8</t>
   </si>
   <si>
-    <t>other</t>
-  </si>
-  <si>
     <t>llewellyn_terminus</t>
   </si>
   <si>
@@ -332,6 +320,42 @@
   </si>
   <si>
     <t>"A02 200" written on sensor and bag. By photo geotag, G04 -&gt; G03 order, and jeremy sensors at 1m, this is not the site at the bottom of the C10 hill</t>
+  </si>
+  <si>
+    <t>on_ice_standard</t>
+  </si>
+  <si>
+    <t>on_ice_intensive</t>
+  </si>
+  <si>
+    <t>on_ice_camp</t>
+  </si>
+  <si>
+    <t>off_ice_standard</t>
+  </si>
+  <si>
+    <t>Venus Mine</t>
+  </si>
+  <si>
+    <t>AB Mountain</t>
+  </si>
+  <si>
+    <t>Carcross Hanger</t>
+  </si>
+  <si>
+    <t>Dail Peak</t>
+  </si>
+  <si>
+    <t>Fraser Wx</t>
+  </si>
+  <si>
+    <t>Klondike  Wx</t>
+  </si>
+  <si>
+    <t>Muffys House</t>
+  </si>
+  <si>
+    <t>Poole Point</t>
   </si>
 </sst>
 </file>
@@ -797,8 +821,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{30214729-FAD1-AB4C-91D6-A2D7E03E2CE5}" name="Table2" displayName="Table2" ref="A1:K47" totalsRowShown="0" headerRowDxfId="11" tableBorderDxfId="10">
-  <autoFilter ref="A1:K47" xr:uid="{30214729-FAD1-AB4C-91D6-A2D7E03E2CE5}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{30214729-FAD1-AB4C-91D6-A2D7E03E2CE5}" name="Table2" displayName="Table2" ref="A1:K56" totalsRowShown="0" headerRowDxfId="11" tableBorderDxfId="10">
+  <autoFilter ref="A1:K56" xr:uid="{30214729-FAD1-AB4C-91D6-A2D7E03E2CE5}"/>
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{D1314852-2294-C84C-828A-C37A76432716}" name="site_type"/>
     <tableColumn id="2" xr3:uid="{57B08370-AE15-194A-9E89-74600FFA2010}" name="site_id" dataDxfId="9"/>
@@ -1133,7 +1157,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{282355AC-F746-9947-AE42-F19047015063}">
-  <dimension ref="A1:K47"/>
+  <dimension ref="A1:K56"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.83203125" customWidth="1"/>
@@ -1153,16 +1177,16 @@
         <v>0</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>34</v>
@@ -1182,7 +1206,7 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>40</v>
+        <v>94</v>
       </c>
       <c r="B2" s="17" t="s">
         <v>1</v>
@@ -1210,12 +1234,12 @@
         <v>26</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>40</v>
+        <v>94</v>
       </c>
       <c r="B3" s="17" t="s">
         <v>2</v>
@@ -1248,7 +1272,7 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>40</v>
+        <v>94</v>
       </c>
       <c r="B4" s="17" t="s">
         <v>3</v>
@@ -1279,7 +1303,7 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>40</v>
+        <v>94</v>
       </c>
       <c r="B5" s="17" t="s">
         <v>4</v>
@@ -1310,7 +1334,7 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>40</v>
+        <v>94</v>
       </c>
       <c r="B6" s="17" t="s">
         <v>5</v>
@@ -1333,13 +1357,13 @@
       <c r="H6" s="11"/>
       <c r="I6" s="5"/>
       <c r="J6" s="12" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="K6" s="8"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>40</v>
+        <v>94</v>
       </c>
       <c r="B7" s="17" t="s">
         <v>6</v>
@@ -1368,7 +1392,7 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>40</v>
+        <v>94</v>
       </c>
       <c r="B8" s="17" t="s">
         <v>7</v>
@@ -1399,7 +1423,7 @@
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>40</v>
+        <v>94</v>
       </c>
       <c r="B9" s="17" t="s">
         <v>8</v>
@@ -1430,7 +1454,7 @@
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>40</v>
+        <v>94</v>
       </c>
       <c r="B10" s="17" t="s">
         <v>9</v>
@@ -1459,7 +1483,7 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>40</v>
+        <v>94</v>
       </c>
       <c r="B11" s="17" t="s">
         <v>10</v>
@@ -1490,7 +1514,7 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>40</v>
+        <v>94</v>
       </c>
       <c r="B12" s="17" t="s">
         <v>11</v>
@@ -1518,12 +1542,12 @@
         <v>26</v>
       </c>
       <c r="K12" s="8" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>40</v>
+        <v>94</v>
       </c>
       <c r="B13" s="17" t="s">
         <v>12</v>
@@ -1554,7 +1578,7 @@
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>40</v>
+        <v>94</v>
       </c>
       <c r="B14" s="17" t="s">
         <v>13</v>
@@ -1585,7 +1609,7 @@
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>40</v>
+        <v>94</v>
       </c>
       <c r="B15" s="17" t="s">
         <v>14</v>
@@ -1616,7 +1640,7 @@
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>40</v>
+        <v>94</v>
       </c>
       <c r="B16" s="17" t="s">
         <v>15</v>
@@ -1647,7 +1671,7 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>40</v>
+        <v>94</v>
       </c>
       <c r="B17" s="17" t="s">
         <v>16</v>
@@ -1678,7 +1702,7 @@
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>40</v>
+        <v>94</v>
       </c>
       <c r="B18" s="17" t="s">
         <v>17</v>
@@ -1709,7 +1733,7 @@
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>40</v>
+        <v>94</v>
       </c>
       <c r="B19" s="17" t="s">
         <v>18</v>
@@ -1740,7 +1764,7 @@
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>40</v>
+        <v>94</v>
       </c>
       <c r="B20" s="17" t="s">
         <v>19</v>
@@ -1771,7 +1795,7 @@
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>40</v>
+        <v>94</v>
       </c>
       <c r="B21" s="17" t="s">
         <v>20</v>
@@ -1802,7 +1826,7 @@
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>40</v>
+        <v>94</v>
       </c>
       <c r="B22" s="17" t="s">
         <v>21</v>
@@ -1833,7 +1857,7 @@
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>40</v>
+        <v>94</v>
       </c>
       <c r="B23" s="17" t="s">
         <v>22</v>
@@ -1864,7 +1888,7 @@
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>40</v>
+        <v>94</v>
       </c>
       <c r="B24" s="17" t="s">
         <v>28</v>
@@ -1895,7 +1919,7 @@
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>40</v>
+        <v>94</v>
       </c>
       <c r="B25" s="17" t="s">
         <v>29</v>
@@ -1926,10 +1950,10 @@
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>40</v>
+        <v>94</v>
       </c>
       <c r="B26" s="17" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C26" s="8" t="s">
         <v>38</v>
@@ -1959,10 +1983,10 @@
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>40</v>
+        <v>94</v>
       </c>
       <c r="B27" s="17" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C27" s="8" t="s">
         <v>38</v>
@@ -1990,7 +2014,7 @@
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>40</v>
+        <v>94</v>
       </c>
       <c r="B28" s="17" t="s">
         <v>30</v>
@@ -2047,10 +2071,10 @@
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>41</v>
+        <v>95</v>
       </c>
       <c r="B31" s="17" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C31" s="8">
         <v>22038781</v>
@@ -2076,10 +2100,10 @@
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>41</v>
+        <v>95</v>
       </c>
       <c r="B32" s="17" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C32" s="8">
         <v>22038779</v>
@@ -2107,10 +2131,10 @@
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>41</v>
+        <v>95</v>
       </c>
       <c r="B33" s="17" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C33" s="8">
         <v>22038776</v>
@@ -2138,10 +2162,10 @@
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>41</v>
+        <v>95</v>
       </c>
       <c r="B34" s="17" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C34" s="8">
         <v>22038777</v>
@@ -2169,10 +2193,10 @@
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>41</v>
+        <v>95</v>
       </c>
       <c r="B35" s="17" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="C35" s="8">
         <v>22038778</v>
@@ -2212,10 +2236,10 @@
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>46</v>
+        <v>96</v>
       </c>
       <c r="B37" s="17" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C37" s="8"/>
       <c r="D37" s="12"/>
@@ -2229,40 +2253,40 @@
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>46</v>
+        <v>96</v>
       </c>
       <c r="B38" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D38" s="13"/>
       <c r="J38" s="15"/>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>46</v>
+        <v>96</v>
       </c>
       <c r="B39" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D39" s="13"/>
       <c r="J39" s="15"/>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
+        <v>96</v>
+      </c>
+      <c r="B40" t="s">
         <v>46</v>
-      </c>
-      <c r="B40" t="s">
-        <v>49</v>
       </c>
       <c r="D40" s="13"/>
       <c r="J40" s="15"/>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>46</v>
+        <v>96</v>
       </c>
       <c r="B41" s="17" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C41" s="8"/>
       <c r="D41" s="14"/>
@@ -2276,57 +2300,237 @@
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>46</v>
+        <v>96</v>
       </c>
       <c r="B42" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D42" s="13"/>
       <c r="J42" s="15"/>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>46</v>
+        <v>96</v>
       </c>
       <c r="B43" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D43" s="13"/>
       <c r="J43" s="15"/>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>46</v>
+        <v>96</v>
       </c>
       <c r="B44" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D44" s="13"/>
       <c r="J44" s="15"/>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>55</v>
+        <v>95</v>
       </c>
       <c r="B46" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="J46" s="15"/>
       <c r="K46" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>55</v>
+        <v>95</v>
       </c>
       <c r="B47" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="J47" s="15"/>
       <c r="K47" t="s">
-        <v>59</v>
-      </c>
+        <v>55</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B48" s="17"/>
+      <c r="C48" s="8"/>
+      <c r="D48" s="8"/>
+      <c r="E48" s="8"/>
+      <c r="F48" s="8"/>
+      <c r="G48" s="9"/>
+      <c r="H48" s="10"/>
+      <c r="I48" s="8"/>
+      <c r="J48" s="10"/>
+      <c r="K48" s="8"/>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>97</v>
+      </c>
+      <c r="B49" s="17" t="s">
+        <v>98</v>
+      </c>
+      <c r="C49" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="D49" s="8">
+        <v>22133684</v>
+      </c>
+      <c r="E49" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="F49" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="G49" s="9"/>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>97</v>
+      </c>
+      <c r="B50" s="17" t="s">
+        <v>99</v>
+      </c>
+      <c r="C50" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="D50" s="8">
+        <v>22133633</v>
+      </c>
+      <c r="E50" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="F50" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="G50" s="9"/>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>97</v>
+      </c>
+      <c r="B51" s="17" t="s">
+        <v>100</v>
+      </c>
+      <c r="C51" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="D51" s="8">
+        <v>22133631</v>
+      </c>
+      <c r="E51" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="F51" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="G51" s="9"/>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>97</v>
+      </c>
+      <c r="B52" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="C52" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="D52" s="8">
+        <v>22133632</v>
+      </c>
+      <c r="E52" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="F52" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="G52" s="9"/>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>97</v>
+      </c>
+      <c r="B53" s="17" t="s">
+        <v>102</v>
+      </c>
+      <c r="C53" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="D53" s="8">
+        <v>22133627</v>
+      </c>
+      <c r="E53" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="F53" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="G53" s="9"/>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>97</v>
+      </c>
+      <c r="B54" s="17" t="s">
+        <v>103</v>
+      </c>
+      <c r="C54" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="D54" s="8">
+        <v>22133678</v>
+      </c>
+      <c r="E54" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="F54" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="G54" s="9"/>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>97</v>
+      </c>
+      <c r="B55" s="17" t="s">
+        <v>104</v>
+      </c>
+      <c r="C55" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="D55" s="8">
+        <v>22133639</v>
+      </c>
+      <c r="E55" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="F55" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="G55" s="9"/>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>97</v>
+      </c>
+      <c r="B56" s="17" t="s">
+        <v>105</v>
+      </c>
+      <c r="C56" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="D56" s="8">
+        <v>22133623</v>
+      </c>
+      <c r="E56" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="F56" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="G56" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2354,36 +2558,36 @@
   <sheetData>
     <row r="1" spans="1:9" s="19" customFormat="1" ht="51" x14ac:dyDescent="0.2">
       <c r="A1" s="19" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B1" s="19" t="s">
+        <v>66</v>
+      </c>
+      <c r="C1" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="D1" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="E1" s="19" t="s">
         <v>70</v>
       </c>
-      <c r="C1" s="19" t="s">
-        <v>88</v>
-      </c>
-      <c r="D1" s="19" t="s">
-        <v>76</v>
-      </c>
-      <c r="E1" s="19" t="s">
-        <v>74</v>
-      </c>
       <c r="F1" s="19" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="G1" s="19" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="H1" s="19" t="s">
         <v>31</v>
       </c>
       <c r="I1" s="19" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B2" s="18">
         <v>45819.666666666664</v>
@@ -2395,32 +2599,32 @@
         <v>22133650</v>
       </c>
       <c r="E2" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="F2" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="G2" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="I2" s="19" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="68" x14ac:dyDescent="0.2">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="51" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="H3" s="19" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I3" s="19" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" ht="68" x14ac:dyDescent="0.2">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B4" s="18">
         <v>45828.711111111108</v>
@@ -2432,21 +2636,21 @@
         <v>22133637</v>
       </c>
       <c r="E4" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="F4" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="G4" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="I4" s="19" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="136" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B5" s="18">
         <v>45831.260416666664</v>
@@ -2458,24 +2662,24 @@
         <v>22133651</v>
       </c>
       <c r="E5" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="F5" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="G5" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="H5" s="19" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="I5" s="19" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="119" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B6" s="18">
         <v>45831.220833333333</v>
@@ -2487,24 +2691,24 @@
         <v>22133670</v>
       </c>
       <c r="E6" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="F6" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="G6" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="H6" s="19" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="I6" s="19" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="51" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B7" s="18">
         <v>45831.220138888886</v>
@@ -2516,19 +2720,19 @@
         <v>22133655</v>
       </c>
       <c r="E7" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="F7" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="G7" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="H7" s="19" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="I7" s="19" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
     </row>
   </sheetData>

</xml_diff>